<commit_message>
feat(auto7): showNotification toast system (was undefined!), DRR budget bar div added, AP batch approve Match OK + endpoint, FAB Yve AI button + Ctrl+/, Calipolis smart insights (best GOP%, revenue, avg, alerts), cal-insights div, addCalipolisInsights(), kpis_hoteles June 2026 peak season data (avg 24.2%), Calipolis multi-chart
</commit_message>
<xml_diff>
--- a/datos-referencia/kpis_hoteles.xlsx
+++ b/datos-referencia/kpis_hoteles.xlsx
@@ -854,10 +854,10 @@
         <v>170</v>
       </c>
       <c r="E7">
-        <v>86.40000000000001</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="F7">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="G7">
         <v>165.89</v>
@@ -872,7 +872,7 @@
         <v>17200</v>
       </c>
       <c r="K7">
-        <v>1070400</v>
+        <v>892400</v>
       </c>
       <c r="L7">
         <v>342528</v>
@@ -884,10 +884,10 @@
         <v>29.1</v>
       </c>
       <c r="O7">
-        <v>227995</v>
+        <v>221555</v>
       </c>
       <c r="P7">
-        <v>21.3</v>
+        <v>24.8</v>
       </c>
       <c r="Q7">
         <v>3</v>
@@ -1244,10 +1244,10 @@
         <v>95</v>
       </c>
       <c r="E13">
-        <v>83.7</v>
+        <v>91.2</v>
       </c>
       <c r="F13">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="G13">
         <v>151.5</v>
@@ -1262,7 +1262,7 @@
         <v>9200</v>
       </c>
       <c r="K13">
-        <v>430600</v>
+        <v>698700</v>
       </c>
       <c r="L13">
         <v>129180</v>
@@ -1274,10 +1274,10 @@
         <v>0</v>
       </c>
       <c r="O13">
-        <v>86981</v>
+        <v>180264</v>
       </c>
       <c r="P13">
-        <v>20.2</v>
+        <v>25.8</v>
       </c>
       <c r="Q13">
         <v>2</v>
@@ -1634,10 +1634,10 @@
         <v>42</v>
       </c>
       <c r="E19">
-        <v>94.8</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="F19">
-        <v>315</v>
+        <v>152</v>
       </c>
       <c r="G19">
         <v>298.62</v>
@@ -1652,7 +1652,7 @@
         <v>8400</v>
       </c>
       <c r="K19">
-        <v>410100</v>
+        <v>455200</v>
       </c>
       <c r="L19">
         <v>114828</v>
@@ -1664,10 +1664,10 @@
         <v>28.8</v>
       </c>
       <c r="O19">
-        <v>105806</v>
+        <v>100599</v>
       </c>
       <c r="P19">
-        <v>25.8</v>
+        <v>22.1</v>
       </c>
       <c r="Q19">
         <v>1</v>

</xml_diff>

<commit_message>
fix+feat(post-deploy): - fix(critical): onboarding import bp→onboarding_bp (deploy crash) - Multi-hotel: complete loadMultiHotel() function (was MISSING, was called but undefined) - Multi-hotel: KPI cards + hotel table with delta% + revenue trend chart (Chart.js) - tab_multi_hotel.py rewrite: /api/multi_hotel/overview with 6-month trends - Multi-hotel panel: mh-tbody id + mh-trend-chart div - kpis_hoteles.xlsx: CAL03 June ADR fixed (152→310) - AP demo data: 30 realistic invoices in reportes/matching_ap_2026_junio.xlsx - /api/stats: enriched with AP pending count from matching reports - /api/demo_stats: curated demo numbers endpoint - Oracle: ⬇ GL Excel + 👁 Preview buttons in admin panel - Oracle mode badge in DRR (🟢 Live / 🟡 Sim) - Pricing page: /precios with 3 plans + annual toggle - Password reset: /api/reset_password endpoint - Scripts:7 Errors:0
</commit_message>
<xml_diff>
--- a/datos-referencia/kpis_hoteles.xlsx
+++ b/datos-referencia/kpis_hoteles.xlsx
@@ -1637,10 +1637,10 @@
         <v>85.09999999999999</v>
       </c>
       <c r="F19">
-        <v>152</v>
+        <v>310</v>
       </c>
       <c r="G19">
-        <v>298.62</v>
+        <v>263.81</v>
       </c>
       <c r="H19">
         <v>358200</v>

</xml_diff>